<commit_message>
Add template Excel, template schema, and example data
</commit_message>
<xml_diff>
--- a/example-data/dummydata-a1.xlsx
+++ b/example-data/dummydata-a1.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="509">
   <si>
     <t>CODE</t>
   </si>
@@ -409,1012 +409,1006 @@
     <t>a1_auteursrechtHouder_1</t>
   </si>
   <si>
-    <t>2000-01-07</t>
+    <t>2005-09-05</t>
+  </si>
+  <si>
+    <t>a1/code/Licentie_4</t>
+  </si>
+  <si>
+    <t>a1_producent_1</t>
+  </si>
+  <si>
+    <t>2030-07-13T11:02:14.997Z</t>
+  </si>
+  <si>
+    <t>a1_taal_1</t>
+  </si>
+  <si>
+    <t>a1_uitgever_1</t>
+  </si>
+  <si>
+    <t>a1_vereisteTijd_1</t>
+  </si>
+  <si>
+    <t>a1_versie_1</t>
+  </si>
+  <si>
+    <t>a1/code/CreatiefWerk_2</t>
+  </si>
+  <si>
+    <t>a1_auteur_2</t>
+  </si>
+  <si>
+    <t>a1_auteursrechtHouder_2</t>
+  </si>
+  <si>
+    <t>2021-07-16</t>
+  </si>
+  <si>
+    <t>a1/code/Licentie_3</t>
+  </si>
+  <si>
+    <t>a1_producent_2</t>
+  </si>
+  <si>
+    <t>2028-12-07T00:37:55.151Z</t>
+  </si>
+  <si>
+    <t>a1_taal_2</t>
+  </si>
+  <si>
+    <t>a1_uitgever_2</t>
+  </si>
+  <si>
+    <t>a1_vereisteTijd_2</t>
+  </si>
+  <si>
+    <t>a1_versie_2</t>
+  </si>
+  <si>
+    <t>a1/code/CreatiefWerk_3</t>
+  </si>
+  <si>
+    <t>a1_auteur_3</t>
+  </si>
+  <si>
+    <t>a1_auteursrechtHouder_3</t>
+  </si>
+  <si>
+    <t>2023-09-22</t>
+  </si>
+  <si>
+    <t>a1_producent_3</t>
+  </si>
+  <si>
+    <t>2015-01-11T07:35:54.620Z</t>
+  </si>
+  <si>
+    <t>a1_taal_3</t>
+  </si>
+  <si>
+    <t>a1_uitgever_3</t>
+  </si>
+  <si>
+    <t>a1_vereisteTijd_3</t>
+  </si>
+  <si>
+    <t>a1_versie_3</t>
+  </si>
+  <si>
+    <t>a1/code/CreatiefWerk_4</t>
+  </si>
+  <si>
+    <t>a1_auteur_4</t>
+  </si>
+  <si>
+    <t>a1_auteursrechtHouder_4</t>
+  </si>
+  <si>
+    <t>2029-10-18</t>
+  </si>
+  <si>
+    <t>a1_producent_4</t>
+  </si>
+  <si>
+    <t>2028-08-30T16:54:37.801Z</t>
+  </si>
+  <si>
+    <t>a1_taal_4</t>
+  </si>
+  <si>
+    <t>a1_uitgever_4</t>
+  </si>
+  <si>
+    <t>a1_vereisteTijd_4</t>
+  </si>
+  <si>
+    <t>a1_versie_4</t>
+  </si>
+  <si>
+    <t>a1/code/CreatiefWerk_5</t>
+  </si>
+  <si>
+    <t>a1_auteur_5|a1_auteur_5b</t>
+  </si>
+  <si>
+    <t>a1_auteursrechtHouder_5|a1_auteursrechtHouder_5b</t>
+  </si>
+  <si>
+    <t>2008-05-04</t>
+  </si>
+  <si>
+    <t>a1/code/Licentie_2|a1/code/Licentie_4</t>
+  </si>
+  <si>
+    <t>a1_producent_5|a1_producent_5b</t>
+  </si>
+  <si>
+    <t>2015-01-08T21:14:13.444Z</t>
+  </si>
+  <si>
+    <t>a1_taal_5|a1_taal_5b</t>
+  </si>
+  <si>
+    <t>a1_uitgever_5|a1_uitgever_5b</t>
+  </si>
+  <si>
+    <t>a1_vereisteTijd_5</t>
+  </si>
+  <si>
+    <t>a1_versie_5</t>
+  </si>
+  <si>
+    <t>bestaatUit</t>
+  </si>
+  <si>
+    <t>bron</t>
+  </si>
+  <si>
+    <t>competentie</t>
+  </si>
+  <si>
+    <t>doelgroep</t>
+  </si>
+  <si>
+    <t>gedefinieerdDoor</t>
+  </si>
+  <si>
+    <t>geldigheid</t>
+  </si>
+  <si>
+    <t>gelijkaardig</t>
+  </si>
+  <si>
+    <t>gerelateerdAan</t>
+  </si>
+  <si>
+    <t>heeftSpecialisatie</t>
+  </si>
+  <si>
+    <t>identificator</t>
+  </si>
+  <si>
+    <t>isBrederDan</t>
+  </si>
+  <si>
+    <t>isLidVan</t>
+  </si>
+  <si>
+    <t>niveau</t>
+  </si>
+  <si>
+    <t>onderwerp</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_1</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_2</t>
+  </si>
+  <si>
+    <t>a1_bron_1</t>
+  </si>
+  <si>
+    <t>a1/code/Doelgroep_5</t>
+  </si>
+  <si>
+    <t>a1_gedefinieerdDoor_1</t>
+  </si>
+  <si>
+    <t>a1_geldigheid_1</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_3</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_5</t>
+  </si>
+  <si>
+    <t>a1/code/Identificator_4</t>
+  </si>
+  <si>
+    <t>a1/code/DoelCollectie_3</t>
+  </si>
+  <si>
+    <t>a1_niveau_1</t>
+  </si>
+  <si>
+    <t>a1_onderwerp_1</t>
+  </si>
+  <si>
+    <t>a1_bron_2</t>
+  </si>
+  <si>
+    <t>a1/code/Doelgroep_2</t>
+  </si>
+  <si>
+    <t>a1_gedefinieerdDoor_2</t>
+  </si>
+  <si>
+    <t>a1_geldigheid_2</t>
+  </si>
+  <si>
+    <t>a1/code/Identificator_3</t>
+  </si>
+  <si>
+    <t>a1/code/DoelCollectie_5</t>
+  </si>
+  <si>
+    <t>a1_niveau_2</t>
+  </si>
+  <si>
+    <t>a1_onderwerp_2</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_4</t>
+  </si>
+  <si>
+    <t>a1_bron_3</t>
+  </si>
+  <si>
+    <t>a1_gedefinieerdDoor_3</t>
+  </si>
+  <si>
+    <t>a1_geldigheid_3</t>
+  </si>
+  <si>
+    <t>a1/code/Identificator_1</t>
+  </si>
+  <si>
+    <t>a1/code/DoelCollectie_4</t>
+  </si>
+  <si>
+    <t>a1_niveau_3</t>
+  </si>
+  <si>
+    <t>a1_onderwerp_3</t>
+  </si>
+  <si>
+    <t>a1_bron_4</t>
+  </si>
+  <si>
+    <t>a1_gedefinieerdDoor_4</t>
+  </si>
+  <si>
+    <t>a1_geldigheid_4</t>
+  </si>
+  <si>
+    <t>a1_niveau_4</t>
+  </si>
+  <si>
+    <t>a1_onderwerp_4</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_1|a1/code/Doel_5</t>
+  </si>
+  <si>
+    <t>a1_bron_5|a1_bron_5b</t>
+  </si>
+  <si>
+    <t>a1/code/Competentie_3|a1/code/Competentie_3</t>
+  </si>
+  <si>
+    <t>a1_gedefinieerdDoor_5|a1_gedefinieerdDoor_5b</t>
+  </si>
+  <si>
+    <t>a1_geldigheid_5</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_5|a1/code/Doel_4</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_5|a1/code/Doel_3</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_1|a1/code/Doel_2</t>
+  </si>
+  <si>
+    <t>a1/code/Identificator_5</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_1|a1/code/Doel_4</t>
+  </si>
+  <si>
+    <t>a1/code/DoelCollectie_2|a1/code/DoelCollectie_5</t>
+  </si>
+  <si>
+    <t>a1_niveau_5|a1_niveau_5b</t>
+  </si>
+  <si>
+    <t>a1_onderwerp_5|a1_onderwerp_5b</t>
+  </si>
+  <si>
+    <t>a1_type_5|a1_type_5b</t>
+  </si>
+  <si>
+    <t>heeftLid</t>
+  </si>
+  <si>
+    <t>a1/code/DoelCollectie_1</t>
+  </si>
+  <si>
+    <t>a1/code/DoelCollectie_2</t>
+  </si>
+  <si>
+    <t>a1_gedefinieerdDoor_5</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_4|a1/code/Doel_5</t>
+  </si>
+  <si>
+    <t>a1_niveau_5</t>
+  </si>
+  <si>
+    <t>leeftijdstype</t>
+  </si>
+  <si>
+    <t>onderwijsniveau</t>
+  </si>
+  <si>
+    <t>a1/code/Doelgroep_1</t>
+  </si>
+  <si>
+    <t>a1_doelgroep_1</t>
+  </si>
+  <si>
+    <t>a1_leeftijdstype_1</t>
+  </si>
+  <si>
+    <t>a1_onderwijsniveau_1</t>
+  </si>
+  <si>
+    <t>a1_doelgroep_2</t>
+  </si>
+  <si>
+    <t>a1_leeftijdstype_2</t>
+  </si>
+  <si>
+    <t>a1_onderwijsniveau_2</t>
+  </si>
+  <si>
+    <t>a1/code/Doelgroep_3</t>
+  </si>
+  <si>
+    <t>a1_doelgroep_3</t>
+  </si>
+  <si>
+    <t>a1_leeftijdstype_3</t>
+  </si>
+  <si>
+    <t>a1_onderwijsniveau_3</t>
+  </si>
+  <si>
+    <t>a1/code/Doelgroep_4</t>
+  </si>
+  <si>
+    <t>a1_doelgroep_4</t>
+  </si>
+  <si>
+    <t>a1_leeftijdstype_4</t>
+  </si>
+  <si>
+    <t>a1_onderwijsniveau_4</t>
+  </si>
+  <si>
+    <t>a1_doelgroep_5|a1_doelgroep_5b</t>
+  </si>
+  <si>
+    <t>a1_leeftijdstype_5|a1_leeftijdstype_5b</t>
+  </si>
+  <si>
+    <t>a1_onderwijsniveau_5|a1_onderwijsniveau_5b</t>
+  </si>
+  <si>
+    <t>valuta</t>
+  </si>
+  <si>
+    <t>a1/code/Geldbedrag_1</t>
+  </si>
+  <si>
+    <t>a1_valuta_1</t>
+  </si>
+  <si>
+    <t>a1/code/Geldbedrag_2</t>
+  </si>
+  <si>
+    <t>a1_valuta_2</t>
+  </si>
+  <si>
+    <t>a1/code/Geldbedrag_3</t>
+  </si>
+  <si>
+    <t>a1_valuta_3</t>
+  </si>
+  <si>
+    <t>a1/code/Geldbedrag_4</t>
+  </si>
+  <si>
+    <t>a1_valuta_4</t>
+  </si>
+  <si>
+    <t>a1/code/Geldbedrag_5</t>
+  </si>
+  <si>
+    <t>a1_valuta_5</t>
+  </si>
+  <si>
+    <t>toegekendDoor</t>
+  </si>
+  <si>
+    <t>a1_toegekendDoor_1</t>
+  </si>
+  <si>
+    <t>a1/code/Identificator_2</t>
+  </si>
+  <si>
+    <t>a1_toegekendDoor_2</t>
+  </si>
+  <si>
+    <t>a1_toegekendDoor_3</t>
+  </si>
+  <si>
+    <t>a1_toegekendDoor_4</t>
+  </si>
+  <si>
+    <t>a1_toegekendDoor_5</t>
+  </si>
+  <si>
+    <t>eenheid</t>
+  </si>
+  <si>
+    <t>waarde</t>
+  </si>
+  <si>
+    <t>a1/code/KwantitatieveWaarde_1</t>
+  </si>
+  <si>
+    <t>a1_eenheid_1</t>
+  </si>
+  <si>
+    <t>a1_waarde_1</t>
+  </si>
+  <si>
+    <t>a1/code/KwantitatieveWaarde_2</t>
+  </si>
+  <si>
+    <t>a1_eenheid_2</t>
+  </si>
+  <si>
+    <t>a1_waarde_2</t>
+  </si>
+  <si>
+    <t>a1/code/KwantitatieveWaarde_3</t>
+  </si>
+  <si>
+    <t>a1_eenheid_3</t>
+  </si>
+  <si>
+    <t>a1_waarde_3</t>
+  </si>
+  <si>
+    <t>a1/code/KwantitatieveWaarde_4</t>
+  </si>
+  <si>
+    <t>a1_eenheid_4</t>
+  </si>
+  <si>
+    <t>a1_waarde_4</t>
+  </si>
+  <si>
+    <t>a1/code/KwantitatieveWaarde_5</t>
+  </si>
+  <si>
+    <t>a1_eenheid_5</t>
+  </si>
+  <si>
+    <t>a1_waarde_5</t>
+  </si>
+  <si>
+    <t>draagtBijAanHetBehalenVan</t>
+  </si>
+  <si>
+    <t>heeftDeel</t>
+  </si>
+  <si>
+    <t>ingerichtDoor</t>
+  </si>
+  <si>
+    <t>isDeelVan</t>
+  </si>
+  <si>
+    <t>leermiddel</t>
+  </si>
+  <si>
+    <t>locatie</t>
+  </si>
+  <si>
+    <t>periode</t>
+  </si>
+  <si>
+    <t>specificatie</t>
+  </si>
+  <si>
+    <t>werklast</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteit_1</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteit_3</t>
+  </si>
+  <si>
+    <t>a1_ingerichtDoor_1</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteit_5</t>
+  </si>
+  <si>
+    <t>a1/code/Leermiddel_4</t>
+  </si>
+  <si>
+    <t>a1_periode_1</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteitspecificatie_1</t>
+  </si>
+  <si>
+    <t>a1_werklast_1</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteit_2</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteit_4</t>
+  </si>
+  <si>
+    <t>a1_ingerichtDoor_2</t>
+  </si>
+  <si>
+    <t>a1/code/Leermiddel_3</t>
+  </si>
+  <si>
+    <t>a1_periode_2</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteitspecificatie_3</t>
+  </si>
+  <si>
+    <t>a1_werklast_2</t>
+  </si>
+  <si>
+    <t>a1_ingerichtDoor_3</t>
+  </si>
+  <si>
+    <t>a1/code/Leermiddel_5</t>
+  </si>
+  <si>
+    <t>a1_periode_3</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteitspecificatie_2</t>
+  </si>
+  <si>
+    <t>a1_werklast_3</t>
+  </si>
+  <si>
+    <t>a1_ingerichtDoor_4</t>
+  </si>
+  <si>
+    <t>a1_periode_4</t>
+  </si>
+  <si>
+    <t>a1_werklast_4</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteit_5|a1/code/Leeractiviteit_5</t>
+  </si>
+  <si>
+    <t>a1_ingerichtDoor_5|a1_ingerichtDoor_5b</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteit_2|a1/code/Leeractiviteit_4</t>
+  </si>
+  <si>
+    <t>a1/code/Leermiddel_1|a1/code/Leermiddel_5</t>
+  </si>
+  <si>
+    <t>a1/code/Adresvoorstelling_2|a1/code/Adresvoorstelling_2</t>
+  </si>
+  <si>
+    <t>a1_periode_5|a1_periode_5b</t>
+  </si>
+  <si>
+    <t>a1_werklast_5</t>
+  </si>
+  <si>
+    <t>contacturen</t>
+  </si>
+  <si>
+    <t>generalisatieVan</t>
+  </si>
+  <si>
+    <t>instructietaal</t>
+  </si>
+  <si>
+    <t>schrijftVoor</t>
+  </si>
+  <si>
+    <t>specialisatieVan</t>
+  </si>
+  <si>
+    <t>a1/code/Openingsurenspecificatie_4</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteitspecificatie_5</t>
+  </si>
+  <si>
+    <t>a1_instructietaal_1</t>
+  </si>
+  <si>
+    <t>a1/code/Openingsurenspecificatie_3</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteitspecificatie_4</t>
+  </si>
+  <si>
+    <t>a1_instructietaal_2</t>
+  </si>
+  <si>
+    <t>a1/code/Leermiddel_1</t>
+  </si>
+  <si>
+    <t>a1_instructietaal_3</t>
+  </si>
+  <si>
+    <t>a1/code/Openingsurenspecificatie_1</t>
+  </si>
+  <si>
+    <t>a1_instructietaal_4</t>
+  </si>
+  <si>
+    <t>a1/code/Leermiddel_2</t>
+  </si>
+  <si>
+    <t>a1/code/Openingsurenspecificatie_1|a1/code/Openingsurenspecificatie_5</t>
+  </si>
+  <si>
+    <t>a1/code/Doel_3|a1/code/Doel_3</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteitspecificatie_5|a1/code/Leeractiviteitspecificatie_4</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteitspecificatie_5|a1/code/Leeractiviteitspecificatie_2</t>
+  </si>
+  <si>
+    <t>a1_instructietaal_5|a1_instructietaal_5b</t>
+  </si>
+  <si>
+    <t>a1/code/Leeractiviteitspecificatie_3|a1/code/Leeractiviteitspecificatie_1</t>
+  </si>
+  <si>
+    <t>a1/code/Leermiddel_1|a1/code/Leermiddel_2</t>
+  </si>
+  <si>
+    <t>benodigdMateriaal</t>
+  </si>
+  <si>
+    <t>dient</t>
+  </si>
+  <si>
+    <t>formaat</t>
+  </si>
+  <si>
+    <t>instructie</t>
+  </si>
+  <si>
+    <t>interactieType</t>
+  </si>
+  <si>
+    <t>kost</t>
+  </si>
+  <si>
+    <t>resultaat</t>
+  </si>
+  <si>
+    <t>sleutelwoord</t>
+  </si>
+  <si>
+    <t>toegankelijkheid</t>
+  </si>
+  <si>
+    <t>vereiste</t>
+  </si>
+  <si>
+    <t>a1_benodigdMateriaal_1</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelElement_5</t>
+  </si>
+  <si>
+    <t>a1_formaat_1</t>
+  </si>
+  <si>
+    <t>a1_instructie_1</t>
+  </si>
+  <si>
+    <t>a1_interactieType_1</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelVerzameling_3</t>
+  </si>
+  <si>
+    <t>a1_resultaat_1</t>
+  </si>
+  <si>
+    <t>a1_sleutelwoord_1</t>
+  </si>
+  <si>
+    <t>a1_toegankelijkheid_1</t>
+  </si>
+  <si>
+    <t>a1_vereiste_1</t>
+  </si>
+  <si>
+    <t>a1_benodigdMateriaal_2</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelElement_2</t>
+  </si>
+  <si>
+    <t>a1_formaat_2</t>
+  </si>
+  <si>
+    <t>a1_instructie_2</t>
+  </si>
+  <si>
+    <t>a1_interactieType_2</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelVerzameling_5</t>
+  </si>
+  <si>
+    <t>a1_resultaat_2</t>
+  </si>
+  <si>
+    <t>a1_sleutelwoord_2</t>
+  </si>
+  <si>
+    <t>a1_toegankelijkheid_2</t>
+  </si>
+  <si>
+    <t>a1_vereiste_2</t>
+  </si>
+  <si>
+    <t>a1_benodigdMateriaal_3</t>
+  </si>
+  <si>
+    <t>a1_formaat_3</t>
+  </si>
+  <si>
+    <t>a1_instructie_3</t>
+  </si>
+  <si>
+    <t>a1_interactieType_3</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelVerzameling_2</t>
+  </si>
+  <si>
+    <t>a1_resultaat_3</t>
+  </si>
+  <si>
+    <t>a1_sleutelwoord_3</t>
+  </si>
+  <si>
+    <t>a1_toegankelijkheid_3</t>
+  </si>
+  <si>
+    <t>a1_vereiste_3</t>
+  </si>
+  <si>
+    <t>a1_benodigdMateriaal_4</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelElement_3</t>
+  </si>
+  <si>
+    <t>a1_formaat_4</t>
+  </si>
+  <si>
+    <t>a1_instructie_4</t>
+  </si>
+  <si>
+    <t>a1_interactieType_4</t>
+  </si>
+  <si>
+    <t>a1_resultaat_4</t>
+  </si>
+  <si>
+    <t>a1_sleutelwoord_4</t>
+  </si>
+  <si>
+    <t>a1_toegankelijkheid_4</t>
+  </si>
+  <si>
+    <t>a1_vereiste_4</t>
+  </si>
+  <si>
+    <t>a1_benodigdMateriaal_5|a1_benodigdMateriaal_5b</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelElement_1|a1/code/LeermiddelElement_5</t>
+  </si>
+  <si>
+    <t>a1/code/Competentie_4|a1/code/Competentie_2</t>
+  </si>
+  <si>
+    <t>a1_formaat_5|a1_formaat_5b</t>
+  </si>
+  <si>
+    <t>a1_instructie_5</t>
+  </si>
+  <si>
+    <t>a1_interactieType_5|a1_interactieType_5b</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelVerzameling_2|a1/code/LeermiddelVerzameling_4</t>
+  </si>
+  <si>
+    <t>a1_resultaat_5|a1_resultaat_5b</t>
+  </si>
+  <si>
+    <t>a1_sleutelwoord_5|a1_sleutelwoord_5b</t>
+  </si>
+  <si>
+    <t>a1_toegankelijkheid_5</t>
+  </si>
+  <si>
+    <t>a1_vereiste_5|a1_vereiste_5b</t>
+  </si>
+  <si>
+    <t>onderdeelVan</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelElement_1</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelElement_4</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelVerzameling_1</t>
+  </si>
+  <si>
+    <t>a1/code/LeermiddelVerzameling_4</t>
+  </si>
+  <si>
+    <t>a1/code/Leermiddel_2|a1/code/Leermiddel_1</t>
   </si>
   <si>
     <t>a1/code/Licentie_1</t>
   </si>
   <si>
-    <t>a1_producent_1</t>
-  </si>
-  <si>
-    <t>2030-01-30T02:05:14.727Z</t>
-  </si>
-  <si>
-    <t>a1_taal_1</t>
-  </si>
-  <si>
-    <t>a1_uitgever_1</t>
-  </si>
-  <si>
-    <t>a1_vereisteTijd_1</t>
-  </si>
-  <si>
-    <t>a1_versie_1</t>
-  </si>
-  <si>
-    <t>a1/code/CreatiefWerk_2</t>
-  </si>
-  <si>
-    <t>a1_auteur_2</t>
-  </si>
-  <si>
-    <t>a1_auteursrechtHouder_2</t>
-  </si>
-  <si>
-    <t>2002-06-07</t>
+    <t>a1/code/Licentie_2</t>
   </si>
   <si>
     <t>a1/code/Licentie_5</t>
   </si>
   <si>
-    <t>a1_producent_2</t>
-  </si>
-  <si>
-    <t>2028-10-03T05:25:17.747Z</t>
-  </si>
-  <si>
-    <t>a1_taal_2</t>
-  </si>
-  <si>
-    <t>a1_uitgever_2</t>
-  </si>
-  <si>
-    <t>a1_vereisteTijd_2</t>
-  </si>
-  <si>
-    <t>a1_versie_2</t>
-  </si>
-  <si>
-    <t>a1/code/CreatiefWerk_3</t>
-  </si>
-  <si>
-    <t>a1_auteur_3</t>
-  </si>
-  <si>
-    <t>a1_auteursrechtHouder_3</t>
-  </si>
-  <si>
-    <t>2020-02-07</t>
-  </si>
-  <si>
-    <t>a1_producent_3</t>
-  </si>
-  <si>
-    <t>2016-08-24T14:57:29.228Z</t>
-  </si>
-  <si>
-    <t>a1_taal_3</t>
-  </si>
-  <si>
-    <t>a1_uitgever_3</t>
-  </si>
-  <si>
-    <t>a1_vereisteTijd_3</t>
-  </si>
-  <si>
-    <t>a1_versie_3</t>
-  </si>
-  <si>
-    <t>a1/code/CreatiefWerk_4</t>
-  </si>
-  <si>
-    <t>a1_auteur_4</t>
-  </si>
-  <si>
-    <t>a1_auteursrechtHouder_4</t>
-  </si>
-  <si>
-    <t>2014-09-15</t>
-  </si>
-  <si>
-    <t>a1/code/Licentie_4</t>
-  </si>
-  <si>
-    <t>a1_producent_4</t>
-  </si>
-  <si>
-    <t>2010-10-02T18:21:01.411Z</t>
-  </si>
-  <si>
-    <t>a1_taal_4</t>
-  </si>
-  <si>
-    <t>a1_uitgever_4</t>
-  </si>
-  <si>
-    <t>a1_vereisteTijd_4</t>
-  </si>
-  <si>
-    <t>a1_versie_4</t>
-  </si>
-  <si>
-    <t>a1/code/CreatiefWerk_5</t>
-  </si>
-  <si>
-    <t>a1_auteur_5|a1_auteur_5b</t>
-  </si>
-  <si>
-    <t>a1_auteursrechtHouder_5|a1_auteursrechtHouder_5b</t>
-  </si>
-  <si>
-    <t>2024-12-17</t>
-  </si>
-  <si>
-    <t>a1/code/Licentie_2|a1/code/Licentie_3</t>
-  </si>
-  <si>
-    <t>a1_producent_5|a1_producent_5b</t>
-  </si>
-  <si>
-    <t>2006-01-20T07:36:31.979Z</t>
-  </si>
-  <si>
-    <t>a1_taal_5|a1_taal_5b</t>
-  </si>
-  <si>
-    <t>a1_uitgever_5|a1_uitgever_5b</t>
-  </si>
-  <si>
-    <t>a1_vereisteTijd_5</t>
-  </si>
-  <si>
-    <t>a1_versie_5</t>
-  </si>
-  <si>
-    <t>bestaatUit</t>
-  </si>
-  <si>
-    <t>bron</t>
-  </si>
-  <si>
-    <t>competentie</t>
-  </si>
-  <si>
-    <t>doelgroep</t>
-  </si>
-  <si>
-    <t>gedefinieerdDoor</t>
-  </si>
-  <si>
-    <t>geldigheid</t>
-  </si>
-  <si>
-    <t>gelijkaardig</t>
-  </si>
-  <si>
-    <t>gerelateerdAan</t>
-  </si>
-  <si>
-    <t>heeftSpecialisatie</t>
-  </si>
-  <si>
-    <t>identificator</t>
-  </si>
-  <si>
-    <t>isBrederDan</t>
-  </si>
-  <si>
-    <t>isLidVan</t>
-  </si>
-  <si>
-    <t>niveau</t>
-  </si>
-  <si>
-    <t>onderwerp</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_1</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_4</t>
-  </si>
-  <si>
-    <t>a1_bron_1</t>
-  </si>
-  <si>
-    <t>a1/code/Doelgroep_2</t>
-  </si>
-  <si>
-    <t>a1_gedefinieerdDoor_1</t>
-  </si>
-  <si>
-    <t>a1_geldigheid_1</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_5</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_2</t>
-  </si>
-  <si>
-    <t>a1/code/Identificator_2</t>
-  </si>
-  <si>
-    <t>a1/code/DoelCollectie_4</t>
-  </si>
-  <si>
-    <t>a1_niveau_1</t>
-  </si>
-  <si>
-    <t>a1_onderwerp_1</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_3</t>
-  </si>
-  <si>
-    <t>a1_bron_2</t>
-  </si>
-  <si>
-    <t>a1_gedefinieerdDoor_2</t>
-  </si>
-  <si>
-    <t>a1_geldigheid_2</t>
-  </si>
-  <si>
-    <t>a1/code/Identificator_4</t>
-  </si>
-  <si>
-    <t>a1/code/DoelCollectie_3</t>
-  </si>
-  <si>
-    <t>a1_niveau_2</t>
-  </si>
-  <si>
-    <t>a1_onderwerp_2</t>
-  </si>
-  <si>
-    <t>a1_bron_3</t>
-  </si>
-  <si>
-    <t>a1_gedefinieerdDoor_3</t>
-  </si>
-  <si>
-    <t>a1_geldigheid_3</t>
-  </si>
-  <si>
-    <t>a1/code/Identificator_5</t>
-  </si>
-  <si>
-    <t>a1/code/DoelCollectie_2</t>
-  </si>
-  <si>
-    <t>a1_niveau_3</t>
-  </si>
-  <si>
-    <t>a1_onderwerp_3</t>
-  </si>
-  <si>
-    <t>a1_bron_4</t>
-  </si>
-  <si>
-    <t>a1/code/Doelgroep_4</t>
-  </si>
-  <si>
-    <t>a1_gedefinieerdDoor_4</t>
-  </si>
-  <si>
-    <t>a1_geldigheid_4</t>
-  </si>
-  <si>
-    <t>a1_niveau_4</t>
-  </si>
-  <si>
-    <t>a1_onderwerp_4</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_2|a1/code/Doel_1</t>
-  </si>
-  <si>
-    <t>a1_bron_5|a1_bron_5b</t>
-  </si>
-  <si>
-    <t>a1/code/Competentie_3|a1/code/Competentie_5</t>
-  </si>
-  <si>
-    <t>a1/code/Doelgroep_5</t>
-  </si>
-  <si>
-    <t>a1_gedefinieerdDoor_5|a1_gedefinieerdDoor_5b</t>
-  </si>
-  <si>
-    <t>a1_geldigheid_5</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_2|a1/code/Doel_4</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_3|a1/code/Doel_4</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_5|a1/code/Doel_2</t>
-  </si>
-  <si>
-    <t>a1/code/Identificator_3</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_3|a1/code/Doel_1</t>
-  </si>
-  <si>
-    <t>a1/code/DoelCollectie_5|a1/code/DoelCollectie_2</t>
-  </si>
-  <si>
-    <t>a1_niveau_5|a1_niveau_5b</t>
-  </si>
-  <si>
-    <t>a1_onderwerp_5|a1_onderwerp_5b</t>
-  </si>
-  <si>
-    <t>a1_type_5|a1_type_5b</t>
-  </si>
-  <si>
-    <t>heeftLid</t>
-  </si>
-  <si>
-    <t>a1/code/DoelCollectie_1</t>
-  </si>
-  <si>
-    <t>a1/code/DoelCollectie_5</t>
-  </si>
-  <si>
-    <t>a1_gedefinieerdDoor_5</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_2|a1/code/Doel_5</t>
-  </si>
-  <si>
-    <t>a1_niveau_5</t>
-  </si>
-  <si>
-    <t>leeftijdstype</t>
-  </si>
-  <si>
-    <t>onderwijsniveau</t>
-  </si>
-  <si>
-    <t>a1/code/Doelgroep_1</t>
-  </si>
-  <si>
-    <t>a1_doelgroep_1</t>
-  </si>
-  <si>
-    <t>a1_leeftijdstype_1</t>
-  </si>
-  <si>
-    <t>a1_onderwijsniveau_1</t>
-  </si>
-  <si>
-    <t>a1_doelgroep_2</t>
-  </si>
-  <si>
-    <t>a1_leeftijdstype_2</t>
-  </si>
-  <si>
-    <t>a1_onderwijsniveau_2</t>
-  </si>
-  <si>
-    <t>a1/code/Doelgroep_3</t>
-  </si>
-  <si>
-    <t>a1_doelgroep_3</t>
-  </si>
-  <si>
-    <t>a1_leeftijdstype_3</t>
-  </si>
-  <si>
-    <t>a1_onderwijsniveau_3</t>
-  </si>
-  <si>
-    <t>a1_doelgroep_4</t>
-  </si>
-  <si>
-    <t>a1_leeftijdstype_4</t>
-  </si>
-  <si>
-    <t>a1_onderwijsniveau_4</t>
-  </si>
-  <si>
-    <t>a1_doelgroep_5|a1_doelgroep_5b</t>
-  </si>
-  <si>
-    <t>a1_leeftijdstype_5|a1_leeftijdstype_5b</t>
-  </si>
-  <si>
-    <t>a1_onderwijsniveau_5|a1_onderwijsniveau_5b</t>
-  </si>
-  <si>
-    <t>valuta</t>
-  </si>
-  <si>
-    <t>a1/code/Geldbedrag_1</t>
-  </si>
-  <si>
-    <t>a1_valuta_1</t>
-  </si>
-  <si>
-    <t>a1/code/Geldbedrag_2</t>
-  </si>
-  <si>
-    <t>a1_valuta_2</t>
-  </si>
-  <si>
-    <t>a1/code/Geldbedrag_3</t>
-  </si>
-  <si>
-    <t>a1_valuta_3</t>
-  </si>
-  <si>
-    <t>a1/code/Geldbedrag_4</t>
-  </si>
-  <si>
-    <t>a1_valuta_4</t>
-  </si>
-  <si>
-    <t>a1/code/Geldbedrag_5</t>
-  </si>
-  <si>
-    <t>a1_valuta_5</t>
-  </si>
-  <si>
-    <t>toegekendDoor</t>
-  </si>
-  <si>
-    <t>a1/code/Identificator_1</t>
-  </si>
-  <si>
-    <t>a1_toegekendDoor_1</t>
-  </si>
-  <si>
-    <t>a1_toegekendDoor_2</t>
-  </si>
-  <si>
-    <t>a1_toegekendDoor_3</t>
-  </si>
-  <si>
-    <t>a1_toegekendDoor_4</t>
-  </si>
-  <si>
-    <t>a1_toegekendDoor_5</t>
-  </si>
-  <si>
-    <t>eenheid</t>
-  </si>
-  <si>
-    <t>waarde</t>
-  </si>
-  <si>
-    <t>a1/code/KwantitatieveWaarde_1</t>
-  </si>
-  <si>
-    <t>a1_eenheid_1</t>
-  </si>
-  <si>
-    <t>a1_waarde_1</t>
-  </si>
-  <si>
-    <t>a1/code/KwantitatieveWaarde_2</t>
-  </si>
-  <si>
-    <t>a1_eenheid_2</t>
-  </si>
-  <si>
-    <t>a1_waarde_2</t>
-  </si>
-  <si>
-    <t>a1/code/KwantitatieveWaarde_3</t>
-  </si>
-  <si>
-    <t>a1_eenheid_3</t>
-  </si>
-  <si>
-    <t>a1_waarde_3</t>
-  </si>
-  <si>
-    <t>a1/code/KwantitatieveWaarde_4</t>
-  </si>
-  <si>
-    <t>a1_eenheid_4</t>
-  </si>
-  <si>
-    <t>a1_waarde_4</t>
-  </si>
-  <si>
-    <t>a1/code/KwantitatieveWaarde_5</t>
-  </si>
-  <si>
-    <t>a1_eenheid_5</t>
-  </si>
-  <si>
-    <t>a1_waarde_5</t>
-  </si>
-  <si>
-    <t>draagtBijAanHetBehalenVan</t>
-  </si>
-  <si>
-    <t>heeftDeel</t>
-  </si>
-  <si>
-    <t>ingerichtDoor</t>
-  </si>
-  <si>
-    <t>isDeelVan</t>
-  </si>
-  <si>
-    <t>leermiddel</t>
-  </si>
-  <si>
-    <t>locatie</t>
-  </si>
-  <si>
-    <t>periode</t>
-  </si>
-  <si>
-    <t>specificatie</t>
-  </si>
-  <si>
-    <t>werklast</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteit_1</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteit_4</t>
-  </si>
-  <si>
-    <t>a1_ingerichtDoor_1</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteit_5</t>
-  </si>
-  <si>
-    <t>a1/code/Leermiddel_3</t>
-  </si>
-  <si>
-    <t>a1_periode_1</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteitspecificatie_2</t>
-  </si>
-  <si>
-    <t>a1_werklast_1</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteit_2</t>
-  </si>
-  <si>
-    <t>a1_ingerichtDoor_2</t>
-  </si>
-  <si>
-    <t>a1/code/Leermiddel_4</t>
-  </si>
-  <si>
-    <t>a1_periode_2</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteitspecificatie_1</t>
-  </si>
-  <si>
-    <t>a1_werklast_2</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteit_3</t>
-  </si>
-  <si>
-    <t>a1_ingerichtDoor_3</t>
-  </si>
-  <si>
-    <t>a1/code/Leermiddel_5</t>
-  </si>
-  <si>
-    <t>a1_periode_3</t>
-  </si>
-  <si>
-    <t>a1_werklast_3</t>
-  </si>
-  <si>
-    <t>a1_ingerichtDoor_4</t>
-  </si>
-  <si>
-    <t>a1_periode_4</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteitspecificatie_3</t>
-  </si>
-  <si>
-    <t>a1_werklast_4</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_1|a1/code/Doel_4</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteit_1|a1/code/Leeractiviteit_4</t>
-  </si>
-  <si>
-    <t>a1_ingerichtDoor_5|a1_ingerichtDoor_5b</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteit_2|a1/code/Leeractiviteit_4</t>
-  </si>
-  <si>
-    <t>a1/code/Leermiddel_2|a1/code/Leermiddel_4</t>
-  </si>
-  <si>
-    <t>a1/code/Adresvoorstelling_2|a1/code/Adresvoorstelling_3</t>
-  </si>
-  <si>
-    <t>a1_periode_5|a1_periode_5b</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteitspecificatie_4</t>
-  </si>
-  <si>
-    <t>a1_werklast_5</t>
-  </si>
-  <si>
-    <t>contacturen</t>
-  </si>
-  <si>
-    <t>generalisatieVan</t>
-  </si>
-  <si>
-    <t>instructietaal</t>
-  </si>
-  <si>
-    <t>schrijftVoor</t>
-  </si>
-  <si>
-    <t>specialisatieVan</t>
-  </si>
-  <si>
-    <t>a1/code/Openingsurenspecificatie_1</t>
-  </si>
-  <si>
-    <t>a1_instructietaal_1</t>
-  </si>
-  <si>
-    <t>a1/code/Leermiddel_2</t>
+    <t>dagVanDeWeek</t>
+  </si>
+  <si>
+    <t>geldigTot</t>
+  </si>
+  <si>
+    <t>geldigVan</t>
+  </si>
+  <si>
+    <t>gesloten</t>
+  </si>
+  <si>
+    <t>open</t>
+  </si>
+  <si>
+    <t>http://example.com/au/dagVanDeWeek_1</t>
+  </si>
+  <si>
+    <t>2027-11-03T01:34:39.990Z</t>
+  </si>
+  <si>
+    <t>2023-07-12T04:43:28.691Z</t>
+  </si>
+  <si>
+    <t>07:25:08</t>
+  </si>
+  <si>
+    <t>09:09:51</t>
+  </si>
+  <si>
+    <t>a1/code/Openingsurenspecificatie_2</t>
+  </si>
+  <si>
+    <t>http://example.com/au/dagVanDeWeek_2</t>
+  </si>
+  <si>
+    <t>2007-01-14T19:00:43.402Z</t>
+  </si>
+  <si>
+    <t>2025-11-16T05:27:55.116Z</t>
+  </si>
+  <si>
+    <t>18:52:10</t>
+  </si>
+  <si>
+    <t>20:56:59</t>
+  </si>
+  <si>
+    <t>http://example.com/au/dagVanDeWeek_3</t>
+  </si>
+  <si>
+    <t>2012-02-07T04:04:22.417Z</t>
+  </si>
+  <si>
+    <t>2029-01-13T17:32:08.166Z</t>
+  </si>
+  <si>
+    <t>11:15:38</t>
+  </si>
+  <si>
+    <t>20:30:00</t>
+  </si>
+  <si>
+    <t>http://example.com/au/dagVanDeWeek_4</t>
+  </si>
+  <si>
+    <t>2013-11-23T09:32:18.638Z</t>
+  </si>
+  <si>
+    <t>2001-07-29T03:54:42.319Z</t>
+  </si>
+  <si>
+    <t>15:25:06</t>
+  </si>
+  <si>
+    <t>17:16:12</t>
   </si>
   <si>
     <t>a1/code/Openingsurenspecificatie_5</t>
   </si>
   <si>
-    <t>a1/code/Leeractiviteitspecificatie_5</t>
-  </si>
-  <si>
-    <t>a1_instructietaal_2</t>
-  </si>
-  <si>
-    <t>a1/code/Leermiddel_1</t>
-  </si>
-  <si>
-    <t>a1_instructietaal_3</t>
-  </si>
-  <si>
-    <t>a1_instructietaal_4</t>
-  </si>
-  <si>
-    <t>a1/code/Openingsurenspecificatie_4|a1/code/Openingsurenspecificatie_2</t>
-  </si>
-  <si>
-    <t>a1/code/Doel_4|a1/code/Doel_3</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteitspecificatie_1|a1/code/Leeractiviteitspecificatie_3</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteitspecificatie_5|a1/code/Leeractiviteitspecificatie_4</t>
-  </si>
-  <si>
-    <t>a1_instructietaal_5|a1_instructietaal_5b</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteitspecificatie_4|a1/code/Leeractiviteitspecificatie_1</t>
-  </si>
-  <si>
-    <t>a1/code/Leermiddel_4|a1/code/Leermiddel_3</t>
-  </si>
-  <si>
-    <t>a1/code/Leeractiviteitspecificatie_3|a1/code/Leeractiviteitspecificatie_3</t>
-  </si>
-  <si>
-    <t>benodigdMateriaal</t>
-  </si>
-  <si>
-    <t>dient</t>
-  </si>
-  <si>
-    <t>formaat</t>
-  </si>
-  <si>
-    <t>instructie</t>
-  </si>
-  <si>
-    <t>interactieType</t>
-  </si>
-  <si>
-    <t>kost</t>
-  </si>
-  <si>
-    <t>resultaat</t>
-  </si>
-  <si>
-    <t>sleutelwoord</t>
-  </si>
-  <si>
-    <t>toegankelijkheid</t>
-  </si>
-  <si>
-    <t>vereiste</t>
-  </si>
-  <si>
-    <t>a1_benodigdMateriaal_1</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelElement_2</t>
-  </si>
-  <si>
-    <t>a1_formaat_1</t>
-  </si>
-  <si>
-    <t>a1_instructie_1</t>
-  </si>
-  <si>
-    <t>a1_interactieType_1</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelVerzameling_1</t>
-  </si>
-  <si>
-    <t>a1_resultaat_1</t>
-  </si>
-  <si>
-    <t>a1_sleutelwoord_1</t>
-  </si>
-  <si>
-    <t>a1_toegankelijkheid_1</t>
-  </si>
-  <si>
-    <t>a1_vereiste_1</t>
-  </si>
-  <si>
-    <t>a1_benodigdMateriaal_2</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelElement_4</t>
-  </si>
-  <si>
-    <t>a1_formaat_2</t>
-  </si>
-  <si>
-    <t>a1_instructie_2</t>
-  </si>
-  <si>
-    <t>a1_interactieType_2</t>
-  </si>
-  <si>
-    <t>a1_resultaat_2</t>
-  </si>
-  <si>
-    <t>a1_sleutelwoord_2</t>
-  </si>
-  <si>
-    <t>a1_toegankelijkheid_2</t>
-  </si>
-  <si>
-    <t>a1_vereiste_2</t>
-  </si>
-  <si>
-    <t>a1_benodigdMateriaal_3</t>
-  </si>
-  <si>
-    <t>a1_formaat_3</t>
-  </si>
-  <si>
-    <t>a1_instructie_3</t>
-  </si>
-  <si>
-    <t>a1_interactieType_3</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelVerzameling_3</t>
-  </si>
-  <si>
-    <t>a1_resultaat_3</t>
-  </si>
-  <si>
-    <t>a1_sleutelwoord_3</t>
-  </si>
-  <si>
-    <t>a1_toegankelijkheid_3</t>
-  </si>
-  <si>
-    <t>a1_vereiste_3</t>
-  </si>
-  <si>
-    <t>a1_benodigdMateriaal_4</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelElement_1</t>
-  </si>
-  <si>
-    <t>a1_formaat_4</t>
-  </si>
-  <si>
-    <t>a1_instructie_4</t>
-  </si>
-  <si>
-    <t>a1_interactieType_4</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelVerzameling_4</t>
-  </si>
-  <si>
-    <t>a1_resultaat_4</t>
-  </si>
-  <si>
-    <t>a1_sleutelwoord_4</t>
-  </si>
-  <si>
-    <t>a1_toegankelijkheid_4</t>
-  </si>
-  <si>
-    <t>a1_vereiste_4</t>
-  </si>
-  <si>
-    <t>a1_benodigdMateriaal_5|a1_benodigdMateriaal_5b</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelElement_5|a1/code/LeermiddelElement_2</t>
-  </si>
-  <si>
-    <t>a1/code/Competentie_4|a1/code/Competentie_5</t>
-  </si>
-  <si>
-    <t>a1_formaat_5|a1_formaat_5b</t>
-  </si>
-  <si>
-    <t>a1_instructie_5</t>
-  </si>
-  <si>
-    <t>a1_interactieType_5|a1_interactieType_5b</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelVerzameling_1|a1/code/LeermiddelVerzameling_5</t>
-  </si>
-  <si>
-    <t>a1_resultaat_5|a1_resultaat_5b</t>
-  </si>
-  <si>
-    <t>a1_sleutelwoord_5|a1_sleutelwoord_5b</t>
-  </si>
-  <si>
-    <t>a1_toegankelijkheid_5</t>
-  </si>
-  <si>
-    <t>a1_vereiste_5|a1_vereiste_5b</t>
-  </si>
-  <si>
-    <t>onderdeelVan</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelElement_3</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelElement_5</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelVerzameling_2</t>
-  </si>
-  <si>
-    <t>a1/code/LeermiddelVerzameling_5</t>
-  </si>
-  <si>
-    <t>a1/code/Leermiddel_3|a1/code/Leermiddel_1</t>
-  </si>
-  <si>
-    <t>a1/code/Licentie_2</t>
-  </si>
-  <si>
-    <t>a1/code/Licentie_3</t>
-  </si>
-  <si>
-    <t>dagVanDeWeek</t>
-  </si>
-  <si>
-    <t>geldigTot</t>
-  </si>
-  <si>
-    <t>geldigVan</t>
-  </si>
-  <si>
-    <t>gesloten</t>
-  </si>
-  <si>
-    <t>open</t>
-  </si>
-  <si>
-    <t>http://example.com/au/dagVanDeWeek_1</t>
-  </si>
-  <si>
-    <t>2019-03-25T14:31:00.372Z</t>
-  </si>
-  <si>
-    <t>2026-02-19T21:18:59.576Z</t>
-  </si>
-  <si>
-    <t>06:19:32</t>
-  </si>
-  <si>
-    <t>03:05:12</t>
-  </si>
-  <si>
-    <t>a1/code/Openingsurenspecificatie_2</t>
-  </si>
-  <si>
-    <t>http://example.com/au/dagVanDeWeek_2</t>
-  </si>
-  <si>
-    <t>2023-04-07T03:34:59.728Z</t>
-  </si>
-  <si>
-    <t>2021-10-12T06:07:50.627Z</t>
-  </si>
-  <si>
-    <t>02:48:34</t>
-  </si>
-  <si>
-    <t>00:04:43</t>
-  </si>
-  <si>
-    <t>a1/code/Openingsurenspecificatie_3</t>
-  </si>
-  <si>
-    <t>http://example.com/au/dagVanDeWeek_3</t>
-  </si>
-  <si>
-    <t>2006-12-10T09:52:00.343Z</t>
-  </si>
-  <si>
-    <t>2021-12-06T12:57:17.549Z</t>
-  </si>
-  <si>
-    <t>05:46:17</t>
-  </si>
-  <si>
-    <t>14:29:45</t>
-  </si>
-  <si>
-    <t>a1/code/Openingsurenspecificatie_4</t>
-  </si>
-  <si>
-    <t>http://example.com/au/dagVanDeWeek_4</t>
-  </si>
-  <si>
-    <t>2026-05-15T05:05:36.260Z</t>
-  </si>
-  <si>
-    <t>2013-07-04T04:01:06.522Z</t>
-  </si>
-  <si>
-    <t>15:56:42</t>
-  </si>
-  <si>
-    <t>10:57:34</t>
-  </si>
-  <si>
     <t>http://example.com/au/dagVanDeWeek_5</t>
   </si>
   <si>
-    <t>2011-11-10T16:32:01.441Z</t>
-  </si>
-  <si>
-    <t>2022-06-22T16:45:36.588Z</t>
-  </si>
-  <si>
-    <t>07:27:40</t>
-  </si>
-  <si>
-    <t>20:53:37</t>
+    <t>2001-03-04T01:44:18.808Z</t>
+  </si>
+  <si>
+    <t>2030-02-24T04:27:30.215Z</t>
+  </si>
+  <si>
+    <t>11:03:08</t>
+  </si>
+  <si>
+    <t>06:47:01</t>
   </si>
   <si>
     <t>tot</t>
@@ -2263,77 +2257,77 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>305</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>306</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>92</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>311</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>312</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>45</v>
       </c>
       <c r="H2" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>313</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>314</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>96</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>316</v>
@@ -2342,7 +2336,7 @@
         <v>317</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>318</v>
@@ -2365,31 +2359,31 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>325</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>314</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>104</v>
@@ -2400,72 +2394,72 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>327</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>328</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>108</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="I6" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>336</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>338</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -2487,28 +2481,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>341</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>344</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>92</v>
@@ -2516,31 +2510,31 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>345</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>314</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>320</v>
+        <v>343</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>347</v>
+        <v>323</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>96</v>
@@ -2548,31 +2542,31 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>314</v>
+        <v>325</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>314</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>351</v>
-      </c>
       <c r="I3" s="1" t="s">
-        <v>320</v>
+        <v>346</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>100</v>
@@ -2580,31 +2574,31 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>352</v>
-      </c>
       <c r="G4" s="1" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>104</v>
@@ -2612,31 +2606,31 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>338</v>
+        <v>320</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>338</v>
+        <v>313</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>320</v>
+        <v>343</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>349</v>
+        <v>325</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>108</v>
@@ -2644,34 +2638,34 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>360</v>
-      </c>
       <c r="I6" s="1" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -2693,235 +2687,235 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="G1" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="L1" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>365</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>367</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>91</v>
       </c>
       <c r="O1" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="P1" s="2" t="s">
-        <v>190</v>
-      </c>
       <c r="Q1" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>368</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>370</v>
       </c>
       <c r="T1" s="2" t="s">
         <v>92</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>94</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H2" s="1" t="s">
+      <c r="J2" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>346</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>377</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>95</v>
       </c>
       <c r="O2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="P2" s="1" t="s">
-        <v>202</v>
-      </c>
       <c r="Q2" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>378</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>380</v>
       </c>
       <c r="T2" s="1" t="s">
         <v>96</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>98</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="H3" s="1" t="s">
+      <c r="J3" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>386</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>377</v>
-      </c>
       <c r="M3" s="1" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>99</v>
       </c>
       <c r="O3" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="P3" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="P3" s="1" t="s">
-        <v>210</v>
-      </c>
       <c r="Q3" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="R3" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>388</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>389</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>100</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>102</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>211</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="H4" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>352</v>
-      </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="L4" s="1" t="s">
-        <v>395</v>
-      </c>
       <c r="M4" s="1" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>103</v>
@@ -2933,149 +2927,149 @@
         <v>217</v>
       </c>
       <c r="Q4" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="R4" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>397</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>398</v>
       </c>
       <c r="T4" s="1" t="s">
         <v>104</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>106</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="H5" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>404</v>
-      </c>
       <c r="L5" s="1" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>107</v>
       </c>
       <c r="O5" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="P5" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="P5" s="1" t="s">
-        <v>223</v>
-      </c>
       <c r="Q5" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="S5" s="1" t="s">
         <v>406</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="S5" s="1" t="s">
-        <v>408</v>
       </c>
       <c r="T5" s="1" t="s">
         <v>108</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>110</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="H6" s="1" t="s">
+      <c r="J6" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>416</v>
-      </c>
       <c r="M6" s="1" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>111</v>
       </c>
       <c r="O6" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="T6" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="P6" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="R6" s="1" t="s">
+      <c r="U6" s="1" t="s">
         <v>418</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>420</v>
       </c>
     </row>
   </sheetData>
@@ -3097,47 +3091,47 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>401</v>
+        <v>420</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>347</v>
+        <v>318</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>422</v>
+        <v>400</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>351</v>
+        <v>318</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>383</v>
+        <v>421</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>423</v>
+        <v>371</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -3159,47 +3153,47 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>377</v>
+        <v>422</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>424</v>
+        <v>394</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>347</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>395</v>
+        <v>375</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>405</v>
+        <v>423</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>318</v>
+        <v>348</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>425</v>
+        <v>385</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -3226,7 +3220,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>127</v>
+        <v>425</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>96</v>
@@ -3234,7 +3228,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>100</v>
@@ -3242,7 +3236,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>428</v>
+        <v>138</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>104</v>
@@ -3250,7 +3244,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>108</v>
@@ -3258,10 +3252,10 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>138</v>
+        <v>427</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -3283,119 +3277,119 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>432</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>437</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>443</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>448</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>453</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>454</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>455</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>348</v>
+        <v>454</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>459</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>461</v>
       </c>
     </row>
   </sheetData>
@@ -3417,65 +3411,65 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>464</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>467</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>470</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>473</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>475</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>476</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>477</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>478</v>
       </c>
     </row>
   </sheetData>
@@ -3494,63 +3488,63 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>481</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>482</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>483</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>490</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>491</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>492</v>
       </c>
       <c r="F4" s="1"/>
     </row>
@@ -3558,13 +3552,13 @@
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="F5" s="1"/>
     </row>
@@ -3572,13 +3566,13 @@
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="F6" s="1"/>
     </row>
@@ -3586,13 +3580,13 @@
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="F7" s="1"/>
     </row>
@@ -3600,13 +3594,13 @@
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="F8" s="1"/>
     </row>
@@ -3626,42 +3620,42 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
   </sheetData>
@@ -3930,60 +3924,60 @@
         <v>158</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -4008,46 +4002,46 @@
         <v>90</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>190</v>
       </c>
       <c r="Q1" s="2" t="s">
         <v>92</v>
@@ -4055,52 +4049,52 @@
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>94</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>196</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>198</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>197</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>202</v>
       </c>
       <c r="Q2" s="1" t="s">
         <v>96</v>
@@ -4108,52 +4102,52 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>98</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="K3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="M3" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="N3" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="P3" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>210</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>100</v>
@@ -4161,22 +4155,22 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>102</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>192</v>
+        <v>210</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>211</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>212</v>
@@ -4185,19 +4179,19 @@
         <v>213</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>214</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>215</v>
@@ -4214,7 +4208,7 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>192</v>
+        <v>210</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>106</v>
@@ -4226,19 +4220,19 @@
         <v>218</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>221</v>
-      </c>
       <c r="I5" s="1" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>191</v>
@@ -4247,19 +4241,19 @@
         <v>191</v>
       </c>
       <c r="L5" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>200</v>
-      </c>
       <c r="O5" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="P5" s="1" t="s">
         <v>222</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>223</v>
       </c>
       <c r="Q5" s="1" t="s">
         <v>108</v>
@@ -4273,49 +4267,49 @@
         <v>110</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="N6" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="P6" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="Q6" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -4337,16 +4331,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>91</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>92</v>
@@ -4354,19 +4348,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>95</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>96</v>
@@ -4374,19 +4368,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>215</v>
+        <v>239</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>99</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>100</v>
@@ -4394,13 +4388,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>212</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>103</v>
@@ -4414,19 +4408,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>107</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>108</v>
@@ -4434,19 +4428,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>241</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>243</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>111</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>112</v>
@@ -4471,83 +4465,83 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>248</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>219</v>
+        <v>256</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>227</v>
+        <v>193</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>262</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -4569,47 +4563,47 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>269</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>271</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>273</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -4631,47 +4625,47 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>276</v>
+        <v>214</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>199</v>
+        <v>276</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>233</v>
+        <v>206</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -4693,65 +4687,65 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>285</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>288</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>291</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>